<commit_message>
Amend text in book 01 Chapter 04
</commit_message>
<xml_diff>
--- a/content-pipeline/inputs/book01/b01_ch04_final.xlsx
+++ b/content-pipeline/inputs/book01/b01_ch04_final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://transre-my.sharepoint.com/personal/fau_transre_com/Documents/_OneDrive/_Operational_Tools/Github/GCSEChinese/Inputs/GCSE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{488A4AFB-25BF-4677-8646-9FA0AE5B38E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36298AA6-6F66-4FF6-A02E-80495B1898E9}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{488A4AFB-25BF-4677-8646-9FA0AE5B38E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3066BC0F-7123-4BC3-91DA-3310F7D60732}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1905" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -215,15 +215,6 @@
     <t>fashionable</t>
   </si>
   <si>
-    <t>＂青年地帶＂——杜絕校園欺凌 
-據報道，民間社工機構引＂青年地帶＂與廣州市海珠區政府合作，向區內十二所學校每校派駐兩名社工。社工在學校主要開展杜絕校園欺凌的活動。＂我們認爲，社工跟教師不一樣，二者是兩種不同的職業。我們會讓學生直接叫我們名字，而不是‘老師’。＂＂青年地帶＂負責人郭欣欣說。 
-項目最初開展時，學校對於社工的作用有懷疑，不過，看到校園欺凌案件接二連三地發生，學校只有抱着試一試的態度。 
-＂每一個孩子都有自己的煩惱，不管是欺凌別人還是被別人欺凌的孩子，他們的家庭一般都有不同的問題，例如父母離婚，單親家庭等等，這些問題導致他們性格出現問題。工作的時候，我們要針對每個孩子的家庭情況和性格特點，對症下藥。＂一位社工告訴記者。
-目前，這12所學校都提供了專門的社工服務場所——社工站。社工站設置有圖書室、桌遊區等，吸引學生在課餘時間前來。午休和放學後是社工站最熱鬧的時候，孩子們有的下棋，有的玩桌遊，更多人在聊天。社工陪他們玩，也陪他們聊天。社工說： ＂很多是他們在課堂上不方便講的話，只要他們願意跟我們說，我們就願意傾聽，併爲他們提供幫助。＂與此同時，社工站還定期召開主題班會，瞭解欺凌背後的根源等等，培養孩子們應對問題，解決矛盾的社交技巧等等。 
-＂目前，國內很多學校都比較避諱校園欺凌話題。郭欣欣說。因此，我們要讓更多的學校看到這個問題，並與社工合作，應對校園欺凌。她透露＂青年地帶＂正在開發一個名爲＂校園零欺凌＂的手機軟件，希望能通過新媒體平臺，增進青少年、家長和教師的互動，共同應對校園欺凌問題。
-http://edu.qq.com</t>
-  </si>
-  <si>
     <t>老土</t>
   </si>
   <si>
@@ -707,6 +698,15 @@
   </si>
   <si>
     <t>對家長來說，這是激勵孩子努力的一種辦法</t>
+  </si>
+  <si>
+    <t>＂青年地帶＂——杜絕校園欺凌 
+據報道，民間社工機構引＂青年地帶＂與廣州市海珠區政府合作，向區內十二所學校每校派駐兩名社工。社工在學校主要開展杜絕校園欺凌的活動。＂我們認爲，社工跟教師不一樣，二者是兩種不同的職業。我們會讓學生直接叫我們名字，而不是‘老師’。＂＂青年地帶＂負責人郭欣欣說。 
+項目最初開展時，學校對於社工的作用有懷疑，不過，看到校園欺凌案件接二連三地發生，學校只有抱着試一試的態度。 
+＂每一個孩子都有自己的煩惱，不管是欺凌別人還是被別人欺凌的孩子，他們的家庭一般都有不同的問題，例如父母離婚，單親家庭等等，這些問題導致他們性格出現問題。工作的時候，我們要針對每個孩子的家庭情況和性格特點，對症下藥。＂一位社工告訴記者。
+目前，這12所學校都提供了專門的社工服務場所——社工站。社工站設置有圖書室、桌遊區等，吸引學生在課餘時間前來。午休和放學後是社工站最熱鬧的時候，孩子們有的下棋，有的玩桌遊，更多人在聊天。社工陪他們玩，也陪他們聊天。社工說： ＂很多是他們在課堂上不方便講的話，只要他們願意跟我們說，我們就願意傾聽，併爲他們提供幫助。＂與此同時，社工站還定期召開主題班會，瞭解欺凌背後的根源等等，培養孩子們應對問題，解決矛盾的社交技巧等等。 
+＂目前，國內很多學校都比較避諱校園欺凌話題。郭欣欣說。因此，我們要讓更多的學校看到這個問題，並與社工合作，應對校園欺凌。她透露＂青年地帶＂正在開發一個名爲＂校園零欺凌＂的手機軟件，希望能通過新媒體平台，增進青少年、家長和教師的互動，共同應對校園欺凌問題。
+http://edu.qq.com</t>
   </si>
 </sst>
 </file>
@@ -792,12 +792,12 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1109,34 +1109,34 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1257,339 +1257,339 @@
     </row>
     <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B6" t="s">
         <v>15</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
         <v>18</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>19</v>
-      </c>
-      <c r="C7" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
         <v>21</v>
-      </c>
-      <c r="C8" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" t="s">
         <v>23</v>
-      </c>
-      <c r="C9" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" t="s">
         <v>25</v>
-      </c>
-      <c r="C10" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" t="s">
         <v>27</v>
-      </c>
-      <c r="C11" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" t="s">
         <v>29</v>
-      </c>
-      <c r="C12" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" t="s">
         <v>31</v>
-      </c>
-      <c r="C13" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" t="s">
         <v>33</v>
-      </c>
-      <c r="C14" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" t="s">
         <v>35</v>
-      </c>
-      <c r="C15" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" t="s">
         <v>37</v>
-      </c>
-      <c r="C16" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" t="s">
         <v>39</v>
-      </c>
-      <c r="C17" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" t="s">
         <v>41</v>
-      </c>
-      <c r="C18" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" t="s">
         <v>43</v>
-      </c>
-      <c r="C19" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" t="s">
         <v>45</v>
-      </c>
-      <c r="C20" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" t="s">
         <v>47</v>
-      </c>
-      <c r="C21" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" t="s">
         <v>49</v>
-      </c>
-      <c r="C22" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" t="s">
         <v>51</v>
-      </c>
-      <c r="C23" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24" t="s">
         <v>53</v>
-      </c>
-      <c r="C24" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" t="s">
         <v>55</v>
-      </c>
-      <c r="C25" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" t="s">
         <v>57</v>
-      </c>
-      <c r="C26" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" t="s">
+        <v>58</v>
+      </c>
+      <c r="C27" t="s">
         <v>59</v>
-      </c>
-      <c r="C27" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" t="s">
+        <v>60</v>
+      </c>
+      <c r="C28" t="s">
         <v>61</v>
-      </c>
-      <c r="C28" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" t="s">
+        <v>62</v>
+      </c>
+      <c r="C29" t="s">
         <v>63</v>
-      </c>
-      <c r="C29" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" t="s">
+        <v>64</v>
+      </c>
+      <c r="C30" t="s">
         <v>65</v>
-      </c>
-      <c r="C30" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" t="s">
+        <v>66</v>
+      </c>
+      <c r="C31" t="s">
         <v>67</v>
-      </c>
-      <c r="C31" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" t="s">
+        <v>68</v>
+      </c>
+      <c r="C32" t="s">
         <v>69</v>
-      </c>
-      <c r="C32" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" t="s">
+        <v>70</v>
+      </c>
+      <c r="C33" t="s">
         <v>71</v>
-      </c>
-      <c r="C33" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" t="s">
+        <v>72</v>
+      </c>
+      <c r="C34" t="s">
         <v>73</v>
-      </c>
-      <c r="C34" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3"/>
       <c r="B35" t="s">
+        <v>74</v>
+      </c>
+      <c r="C35" t="s">
         <v>75</v>
-      </c>
-      <c r="C35" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3"/>
       <c r="B36" t="s">
+        <v>76</v>
+      </c>
+      <c r="C36" t="s">
         <v>77</v>
-      </c>
-      <c r="C36" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>
       <c r="B37" t="s">
+        <v>78</v>
+      </c>
+      <c r="C37" t="s">
         <v>79</v>
-      </c>
-      <c r="C37" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
       <c r="B38" t="s">
+        <v>80</v>
+      </c>
+      <c r="C38" t="s">
         <v>81</v>
-      </c>
-      <c r="C38" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
       <c r="B39" t="s">
+        <v>82</v>
+      </c>
+      <c r="C39" t="s">
         <v>83</v>
-      </c>
-      <c r="C39" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3"/>
       <c r="B40" t="s">
+        <v>84</v>
+      </c>
+      <c r="C40" t="s">
         <v>85</v>
-      </c>
-      <c r="C40" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3"/>
       <c r="B41" t="s">
+        <v>86</v>
+      </c>
+      <c r="C41" t="s">
         <v>87</v>
-      </c>
-      <c r="C41" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3"/>
       <c r="B42" t="s">
+        <v>88</v>
+      </c>
+      <c r="C42" t="s">
         <v>89</v>
-      </c>
-      <c r="C42" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1634,33 +1634,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>102</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1671,10 +1671,10 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D4" t="s">
         <v>104</v>
-      </c>
-      <c r="D4" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1685,10 +1685,10 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1699,10 +1699,10 @@
         <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1713,528 +1713,528 @@
         <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D7" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
         <v>16</v>
       </c>
-      <c r="B8" t="s">
-        <v>17</v>
-      </c>
       <c r="C8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D8" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" t="s">
         <v>21</v>
       </c>
-      <c r="B9" t="s">
-        <v>22</v>
-      </c>
       <c r="C9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
         <v>19</v>
       </c>
-      <c r="B10" t="s">
-        <v>20</v>
-      </c>
       <c r="C10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s">
         <v>23</v>
       </c>
-      <c r="B11" t="s">
-        <v>24</v>
-      </c>
       <c r="C11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" t="s">
         <v>25</v>
       </c>
-      <c r="B12" t="s">
-        <v>26</v>
-      </c>
       <c r="C12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D12" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" t="s">
         <v>27</v>
       </c>
-      <c r="B13" t="s">
-        <v>28</v>
-      </c>
       <c r="C13" t="s">
+        <v>113</v>
+      </c>
+      <c r="D13" t="s">
         <v>114</v>
-      </c>
-      <c r="D13" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" t="s">
         <v>29</v>
       </c>
-      <c r="B14" t="s">
-        <v>30</v>
-      </c>
       <c r="C14" t="s">
+        <v>115</v>
+      </c>
+      <c r="D14" t="s">
         <v>116</v>
-      </c>
-      <c r="D14" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" t="s">
         <v>33</v>
       </c>
-      <c r="B15" t="s">
-        <v>34</v>
-      </c>
       <c r="C15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D15" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" t="s">
         <v>31</v>
       </c>
-      <c r="B16" t="s">
-        <v>32</v>
-      </c>
       <c r="C16" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D16" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" t="s">
         <v>35</v>
       </c>
-      <c r="B17" t="s">
-        <v>36</v>
-      </c>
       <c r="C17" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D17" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" t="s">
         <v>39</v>
       </c>
-      <c r="B18" t="s">
-        <v>40</v>
-      </c>
       <c r="C18" t="s">
+        <v>120</v>
+      </c>
+      <c r="D18" t="s">
         <v>121</v>
-      </c>
-      <c r="D18" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" t="s">
         <v>41</v>
       </c>
-      <c r="B19" t="s">
-        <v>42</v>
-      </c>
       <c r="C19" t="s">
+        <v>122</v>
+      </c>
+      <c r="D19" t="s">
         <v>123</v>
-      </c>
-      <c r="D19" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" t="s">
         <v>43</v>
       </c>
-      <c r="B20" t="s">
-        <v>44</v>
-      </c>
       <c r="C20" t="s">
+        <v>124</v>
+      </c>
+      <c r="D20" t="s">
         <v>125</v>
-      </c>
-      <c r="D20" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" t="s">
         <v>37</v>
       </c>
-      <c r="B21" t="s">
-        <v>38</v>
-      </c>
       <c r="C21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D21" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>48</v>
+      </c>
+      <c r="B22" t="s">
         <v>49</v>
       </c>
-      <c r="B22" t="s">
-        <v>50</v>
-      </c>
       <c r="C22" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D22" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>46</v>
+      </c>
+      <c r="B23" t="s">
         <v>47</v>
       </c>
-      <c r="B23" t="s">
-        <v>48</v>
-      </c>
       <c r="C23" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D23" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24" t="s">
         <v>45</v>
       </c>
-      <c r="B24" t="s">
-        <v>46</v>
-      </c>
       <c r="C24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D24" t="s">
         <v>130</v>
-      </c>
-      <c r="D24" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>50</v>
+      </c>
+      <c r="B25" t="s">
         <v>51</v>
       </c>
-      <c r="B25" t="s">
-        <v>52</v>
-      </c>
       <c r="C25" t="s">
+        <v>131</v>
+      </c>
+      <c r="D25" t="s">
         <v>132</v>
-      </c>
-      <c r="D25" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B26" t="s">
         <v>53</v>
       </c>
-      <c r="B26" t="s">
-        <v>54</v>
-      </c>
       <c r="C26" t="s">
+        <v>133</v>
+      </c>
+      <c r="D26" t="s">
         <v>134</v>
-      </c>
-      <c r="D26" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" t="s">
         <v>55</v>
       </c>
-      <c r="B27" t="s">
-        <v>56</v>
-      </c>
       <c r="C27" t="s">
+        <v>135</v>
+      </c>
+      <c r="D27" t="s">
         <v>136</v>
-      </c>
-      <c r="D27" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" t="s">
         <v>57</v>
       </c>
-      <c r="B28" t="s">
-        <v>58</v>
-      </c>
       <c r="C28" t="s">
+        <v>137</v>
+      </c>
+      <c r="D28" t="s">
         <v>138</v>
-      </c>
-      <c r="D28" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>58</v>
+      </c>
+      <c r="B29" t="s">
         <v>59</v>
       </c>
-      <c r="B29" t="s">
-        <v>60</v>
-      </c>
       <c r="C29" t="s">
+        <v>139</v>
+      </c>
+      <c r="D29" t="s">
         <v>140</v>
-      </c>
-      <c r="D29" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>60</v>
+      </c>
+      <c r="B30" t="s">
         <v>61</v>
       </c>
-      <c r="B30" t="s">
-        <v>62</v>
-      </c>
       <c r="C30" t="s">
+        <v>141</v>
+      </c>
+      <c r="D30" t="s">
         <v>142</v>
-      </c>
-      <c r="D30" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>62</v>
+      </c>
+      <c r="B31" t="s">
         <v>63</v>
       </c>
-      <c r="B31" t="s">
-        <v>64</v>
-      </c>
       <c r="C31" t="s">
+        <v>143</v>
+      </c>
+      <c r="D31" t="s">
         <v>144</v>
-      </c>
-      <c r="D31" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B32" t="s">
         <v>65</v>
       </c>
-      <c r="B32" t="s">
-        <v>66</v>
-      </c>
       <c r="C32" t="s">
-        <v>146</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>167</v>
+        <v>145</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>66</v>
+      </c>
+      <c r="B33" t="s">
         <v>67</v>
       </c>
-      <c r="B33" t="s">
-        <v>68</v>
-      </c>
       <c r="C33" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D33" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>68</v>
+      </c>
+      <c r="B34" t="s">
         <v>69</v>
       </c>
-      <c r="B34" t="s">
-        <v>70</v>
-      </c>
       <c r="C34" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D34" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>70</v>
+      </c>
+      <c r="B35" t="s">
         <v>71</v>
       </c>
-      <c r="B35" t="s">
-        <v>72</v>
-      </c>
       <c r="C35" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D35" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>72</v>
+      </c>
+      <c r="B36" t="s">
         <v>73</v>
       </c>
-      <c r="B36" t="s">
-        <v>74</v>
-      </c>
       <c r="C36" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>74</v>
+      </c>
+      <c r="B37" t="s">
         <v>75</v>
       </c>
-      <c r="B37" t="s">
-        <v>76</v>
-      </c>
       <c r="C37" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D37" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>76</v>
+      </c>
+      <c r="B38" t="s">
         <v>77</v>
       </c>
-      <c r="B38" t="s">
-        <v>78</v>
-      </c>
       <c r="C38" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D38" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>78</v>
+      </c>
+      <c r="B39" t="s">
         <v>79</v>
       </c>
-      <c r="B39" t="s">
-        <v>80</v>
-      </c>
       <c r="C39" t="s">
+        <v>152</v>
+      </c>
+      <c r="D39" t="s">
         <v>153</v>
-      </c>
-      <c r="D39" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>80</v>
+      </c>
+      <c r="B40" t="s">
         <v>81</v>
       </c>
-      <c r="B40" t="s">
-        <v>82</v>
-      </c>
       <c r="C40" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D40" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>82</v>
+      </c>
+      <c r="B41" t="s">
         <v>83</v>
       </c>
-      <c r="B41" t="s">
-        <v>84</v>
-      </c>
       <c r="C41" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D41" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>84</v>
+      </c>
+      <c r="B42" t="s">
         <v>85</v>
       </c>
-      <c r="B42" t="s">
-        <v>86</v>
-      </c>
       <c r="C42" t="s">
+        <v>156</v>
+      </c>
+      <c r="D42" t="s">
         <v>157</v>
-      </c>
-      <c r="D42" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>86</v>
+      </c>
+      <c r="B43" t="s">
         <v>87</v>
       </c>
-      <c r="B43" t="s">
-        <v>88</v>
-      </c>
       <c r="C43" t="s">
+        <v>158</v>
+      </c>
+      <c r="D43" t="s">
         <v>159</v>
-      </c>
-      <c r="D43" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>88</v>
+      </c>
+      <c r="B44" t="s">
         <v>89</v>
       </c>
-      <c r="B44" t="s">
-        <v>90</v>
-      </c>
       <c r="C44" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D44" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>